<commit_message>
Lista de corte: columna 条码 con el código de barras limpio para la etiqueta de AutoCUT (Python y web de curvado, 6/6 iguales)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WJ5waVG7DhvphWW3Sx2Zp5
</commit_message>
<xml_diff>
--- a/PENDRIVE/4_ALACENA_SPAR/lista_corte.xlsx
+++ b/PENDRIVE/4_ALACENA_SPAR/lista_corte.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X12"/>
+  <dimension ref="A1:Y12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -440,6 +440,7 @@
     <col width="8" customWidth="1" min="22" max="22"/>
     <col width="6" customWidth="1" min="23" max="23"/>
     <col width="40" customWidth="1" min="24" max="24"/>
+    <col width="15" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -563,6 +564,11 @@
           <t>部件名称</t>
         </is>
       </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>条码</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -647,6 +653,11 @@
       <c r="X2" t="inlineStr">
         <is>
           <t>ALACENA-SPAR_Alacena Spar_Techo</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>9992610010016</t>
         </is>
       </c>
     </row>
@@ -735,6 +746,11 @@
           <t>ALACENA-SPAR_Alacena Spar_Lateral der</t>
         </is>
       </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>9992610010023</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -821,6 +837,11 @@
           <t>ALACENA-SPAR_Alacena Spar_Lateral izq</t>
         </is>
       </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>9992610010030</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -907,6 +928,11 @@
           <t>ALACENA-SPAR_Alacena Spar_Tapa inferior</t>
         </is>
       </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>9992610010047</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -993,6 +1019,11 @@
           <t>ALACENA-SPAR_Alacena Spar_Liston frente</t>
         </is>
       </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>9992610010054</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1079,6 +1110,11 @@
           <t>ALACENA-SPAR_Alacena Spar_Liston atras</t>
         </is>
       </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>9992610010061</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1165,6 +1201,11 @@
           <t>ALACENA-SPAR_Alacena Spar_Estante</t>
         </is>
       </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>9992610010078</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1251,6 +1292,11 @@
           <t>ALACENA-SPAR_Alacena Spar_Fondo</t>
         </is>
       </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>9992610010085</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1337,6 +1383,11 @@
           <t>ALACENA-SPAR_Alacena Spar_Puerta der</t>
         </is>
       </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>9992610010092</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1423,6 +1474,11 @@
           <t>ALACENA-SPAR_Alacena Spar_Puerta izq</t>
         </is>
       </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>9992610010108</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1507,6 +1563,11 @@
       <c r="X12" t="inlineStr">
         <is>
           <t>ALACENA-SPAR_Alacena Spar_Puerta rebatible</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>9992610010115</t>
         </is>
       </c>
     </row>

</xml_diff>